<commit_message>
Keep shape picture fills, hyperlinks and drawing order
Relationships a shape uses are stored with it (rels: hyperlink target, or
a picture fill saved in data/media/) and recreated on import; layer keeps
the number of pictures and charts drawn below the shape. Only form controls
and links to parts that are not exported still produce a warning. diff
pairs shapes by name and compares them independently of ids.

Example 08-shapes gains a shape behind the picture, a hyperlinked shape and
a picture fill.

Also: zero outlineLevelRow/Col (LibreOffice) no longer cause a false
verify difference; README links are absolute so they work on PyPI, with the
exact trusted-publisher settings; Changelog URL in the package metadata.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019UZs6wsi5TT3GKqgC7bYeY
</commit_message>
<xml_diff>
--- a/examples/08-shapes.xlsx
+++ b/examples/08-shapes.xlsx
@@ -127,6 +127,54 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="Frame 8"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="305496"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>Behind the picture</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -152,7 +200,7 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
-  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
@@ -204,7 +252,7 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
@@ -252,7 +300,7 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
@@ -300,7 +348,7 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
@@ -339,7 +387,7 @@
     </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
@@ -434,12 +482,110 @@
     </xdr:grpSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="Link 9">
+          <a:hlinkClick r:id="rId2"/>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="DDEBF7"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="305496"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>Project page</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="Picture fill 10"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:blipFill>
+          <a:blip r:embed="rId3"/>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </a:blipFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="305496"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </wsDr>
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>

</xml_diff>